<commit_message>
Scope rewards to tiles and areas (HLR-9); Rewards tab mirrors Areas
- BFF: rewards get a tile, optional area and match mode (selected tasks
  or all tasks in scope); tags must be in scope; narrowing asks before
  untagging; deleting an area widens its rewards to the tile; deleting a
  tile removes its rewards. Migration 0003_reward_scope infers scope from
  existing tags and marks the rest "Needs a tile", with no data loss
- New endpoints/filters: GET /areas/{id}/rewards, /rewards?categoryId&areaId;
  task detail says whether each reward counts it by tag or by scope
- MFE: Rewards tab navigates tiles -> tile -> area like the Areas tab, with
  the same tile and area editing (shared components in manage.jsx);
  "Rewards you can earn here" on area screens; scoped tagging on tasks
- Docs and workbook: HLR-9 marked built; 59 tests pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rewards/Rewards_HLRD_LLRD.xlsx
+++ b/docs/rewards/Rewards_HLRD_LLRD.xlsx
@@ -1129,7 +1129,7 @@
     <col width="37" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Before HLR-9 build</t>
+          <t>Built with "no" (HLR-9); revisit after real use</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
     <row r="91">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>Reward scope and matching (HLR-9) ⏳ next</t>
+          <t>Reward scope and matching (HLR-9) ✅</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3370,7 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3416,12 +3416,12 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Each reward card shows its scope as a breadcrumb (e.g. "Household › Kitchen" or "Fun") and its match mode. The rewards list can be filtered by tile and by area, in addition to status</t>
+          <t>Each reward card shows its scope as a breadcrumb (e.g. "Household › Kitchen" or "Fun") and its match mode. The Rewards tab is navigated like the Areas tab: tile cards (with active / to-claim / claimed counts) → a tile (its whole-tile rewards, then one row per area) → an area (its rewards, plus whole-tile rewards that also count there). Each level filters by status and has + New reward preset to that tile or area</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>⏳</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4365,12 +4365,12 @@
       </c>
       <c r="B175" s="7" t="inlineStr">
         <is>
-          <t>Reward create/update accept categoryId (required on create), areaId (optional) and match (selected | all_in_scope); reward responses include scope {categoryId, categoryName, areaId, areaName}, match and needsTile</t>
+          <t>Reward create/update accept categoryId (required on create), areaId (optional; null = whole tile) and matchMode (selected | all); update also accepts untagOutside (narrowing answers 409 listing the tasks until it's true). Reward responses include categoryId, categoryName, categoryIcon, areaId, areaName, matchMode, needsTile and matchedTaskCount</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr">
         <is>
-          <t>⏳ (HLR-9)</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="C176" s="7" t="inlineStr">
         <is>
-          <t>⏳ (HLR-9)</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -9266,12 +9266,12 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Each reward card shows its scope as a breadcrumb (e.g. "Household › Kitchen" or "Fun") and its match mode. The rewards list can be filtered by tile and by area, in addition to status</t>
+          <t>Each reward card shows its scope as a breadcrumb (e.g. "Household › Kitchen" or "Fun") and its match mode. The Rewards tab is navigated like the Areas tab: tile cards (with active / to-claim / claimed counts) → a tile (its whole-tile rewards, then one row per area) → an area (its rewards, plus whole-tile rewards that also count there). Each level filters by status and has + New reward preset to that tile or area</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -9359,7 +9359,7 @@
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -9403,7 +9403,7 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -9491,7 +9491,7 @@
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
@@ -11026,12 +11026,12 @@
       </c>
       <c r="D111" s="8" t="inlineStr">
         <is>
-          <t>Reward create/update accept categoryId (required on create), areaId (optional) and match (selected | all_in_scope); reward responses include scope {categoryId, categoryName, areaId, areaName}, match and needsTile</t>
+          <t>Reward create/update accept categoryId (required on create), areaId (optional; null = whole tile) and matchMode (selected | all); update also accepts untagOutside (narrowing answers 409 listing the tasks until it's true). Reward responses include categoryId, categoryName, categoryIcon, areaId, areaName, matchMode, needsTile and matchedTaskCount</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F111" s="8" t="inlineStr">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F112" s="8" t="inlineStr">
@@ -13319,7 +13319,7 @@
       </c>
       <c r="E163" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F163" s="8" t="inlineStr">
@@ -13363,7 +13363,7 @@
       </c>
       <c r="E164" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F164" s="8" t="inlineStr">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="E165" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F165" s="8" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="E166" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F166" s="8" t="inlineStr">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="E167" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F167" s="8" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_reward_scope_validation, test_tagging_outside_scope_rejected, test_narrowing_scope_untags</t>
+          <t>test_reward_scope_validation, test_tagging_outside_scope_rejected, test_narrowing_scope_untags</t>
         </is>
       </c>
     </row>
@@ -14970,7 +14970,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_all_in_scope_counts_untagged_and_new_tasks, test_other_tile_never_counts</t>
+          <t>test_all_in_scope_counts_untagged_and_new_tasks, test_other_tile_never_counts</t>
         </is>
       </c>
     </row>
@@ -14987,7 +14987,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_area_lists_matching_rewards, test_task_detail_lists_matching_rewards</t>
+          <t>test_area_lists_matching_rewards, test_task_detail_lists_matching_rewards</t>
         </is>
       </c>
     </row>
@@ -15004,7 +15004,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_deleting_area_widens_reward_scope</t>
+          <t>test_deleting_area_widens_reward_scope</t>
         </is>
       </c>
     </row>
@@ -15033,12 +15033,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>migration 0002_reward_scope</t>
+          <t>migration 0003_reward_scope</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_migration_infers_scope_and_keeps_data (runs against a pre-migration fixture database)</t>
+          <t>test_migration_infers_scope_and_keeps_data (runs against a database at 0002_details), test_needs_a_tile_reward_must_pick_one_first, test_claimed_reward_without_a_tile_can_still_get_one</t>
         </is>
       </c>
     </row>
@@ -17035,12 +17035,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Reward scope and matching (HLR-9), shipped as the first data-preserving migration</t>
+          <t>Reward scope and matching (HLR-9), shipped as a data-preserving migration (0003_reward_scope)</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>⏳ next, after T3a</t>
+          <t>✅ (branch)</t>
         </is>
       </c>
     </row>
@@ -17585,7 +17585,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add task planning and visibility (HLR-11)
- Tasks: milestone, announce/silent, due date/time and days to complete
  (all optional and independent); migration 0004_task_planning defaults
  existing tasks with no data loss
- Overdue flag; area list filters for milestones and due (overdue, today,
  this week) and sort by due date
- Reward rule "Milestone completed": unlocks when all linked milestones
  are done (0 of 0 never unlocks)
- Completion: announced tasks celebrate with a WhatsApp share prompt,
  milestones get a bigger celebration, silent tasks are only "Logged"
- UI: More options on the add form, Planning card and Day X of N on task
  detail, plan chips on task rows
- Dashboard: Overdue KPI and Milestones table
- Docs and workbook updated; 64 tests pass. Hiding silent tasks from
  visitors comes with the owner passcode (hosting)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rewards/Rewards_HLRD_LLRD.xlsx
+++ b/docs/rewards/Rewards_HLRD_LLRD.xlsx
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Before HLR-11 build</t>
+          <t>Built with all (HLR-11); revisit after real use</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅ (hiding silent tasks from visitors comes with the passcode)</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
     <row r="218">
       <c r="A218" s="13" t="inlineStr">
         <is>
-          <t>LLR-11 Task planning and visibility (HLR-11) ⏳ next</t>
+          <t>LLR-11 Task planning and visibility (HLR-11) ✅</t>
         </is>
       </c>
     </row>
@@ -4886,7 +4886,7 @@
     <row r="221">
       <c r="A221" s="13" t="inlineStr">
         <is>
-          <t>LLR-11 Task planning and visibility (HLR-11) ⏳ next</t>
+          <t>LLR-11 Task planning and visibility (HLR-11) ✅</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="C223" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4932,12 +4932,12 @@
       </c>
       <c r="B224" s="7" t="inlineStr">
         <is>
-          <t>Milestones show a 🏁 badge on task rows and task detail. The area task list has a Milestones only filter, and the dashboard has a *Milestones* table (title, tile › area, due, done / overdue / upcoming)</t>
+          <t>Milestones show a 🏁 badge on task rows (area list, Tasks list, Link screen) and task detail. The area task list has a Milestones only filter, and the dashboard has a *Milestones* table (title, tile › area, due, done / overdue / upcoming)</t>
         </is>
       </c>
       <c r="C224" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="C225" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4966,12 +4966,12 @@
       </c>
       <c r="B226" s="7" t="inlineStr">
         <is>
-          <t>New reward rule Milestone completed (alongside *N completions* and *streak of N*). The reward unlocks when every milestone task it matches has at least one completion (BR-R25). Creating one that matches no milestone task is rejected (422)</t>
+          <t>New reward rule Milestone completed (alongside *N completions* and *streak of N*). The reward unlocks when every milestone task linked to it has at least one completion (BR-R25). With no milestone linked yet it shows 0 of 0 and never unlocks (tasks are linked later, on the Link screen)</t>
         </is>
       </c>
       <c r="C226" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="C227" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="C228" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>🟡 🔕 marker and quiet completion built; hiding from visitors comes with the owner passcode (hosting)</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="C229" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C230" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="C231" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="C232" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="C233" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
       </c>
       <c r="C234" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
       </c>
       <c r="C235" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F117" s="8" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F131" s="8" t="inlineStr">
@@ -11967,12 +11967,12 @@
       </c>
       <c r="D132" s="8" t="inlineStr">
         <is>
-          <t>Milestones show a 🏁 badge on task rows and task detail. The area task list has a Milestones only filter, and the dashboard has a *Milestones* table (title, tile › area, due, done / overdue / upcoming)</t>
+          <t>Milestones show a 🏁 badge on task rows (area list, Tasks list, Link screen) and task detail. The area task list has a Milestones only filter, and the dashboard has a *Milestones* table (title, tile › area, due, done / overdue / upcoming)</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F132" s="8" t="inlineStr">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F133" s="8" t="inlineStr">
@@ -12055,12 +12055,12 @@
       </c>
       <c r="D134" s="8" t="inlineStr">
         <is>
-          <t>New reward rule Milestone completed (alongside *N completions* and *streak of N*). The reward unlocks when every milestone task it matches has at least one completion (BR-R25). Creating one that matches no milestone task is rejected (422)</t>
+          <t>New reward rule Milestone completed (alongside *N completions* and *streak of N*). The reward unlocks when every milestone task linked to it has at least one completion (BR-R25). With no milestone linked yet it shows 0 of 0 and never unlocks (tasks are linked later, on the Link screen)</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F134" s="8" t="inlineStr">
@@ -12104,7 +12104,7 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
@@ -12148,7 +12148,7 @@
       </c>
       <c r="E136" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built (manual test)</t>
         </is>
       </c>
       <c r="F136" s="8" t="inlineStr">
@@ -12192,7 +12192,7 @@
       </c>
       <c r="E137" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F137" s="8" t="inlineStr">
@@ -12236,7 +12236,7 @@
       </c>
       <c r="E138" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F138" s="8" t="inlineStr">
@@ -12280,7 +12280,7 @@
       </c>
       <c r="E139" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F139" s="8" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="E140" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F140" s="8" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="E141" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F141" s="8" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="E142" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F142" s="8" t="inlineStr">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="E143" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F143" s="8" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="E174" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F174" s="8" t="inlineStr">
@@ -13864,7 +13864,7 @@
       </c>
       <c r="E175" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F175" s="8" t="inlineStr">
@@ -13908,7 +13908,7 @@
       </c>
       <c r="E176" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F176" s="8" t="inlineStr">
@@ -13952,7 +13952,7 @@
       </c>
       <c r="E177" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F177" s="8" t="inlineStr">
@@ -13996,7 +13996,7 @@
       </c>
       <c r="E178" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F178" s="8" t="inlineStr">
@@ -14810,7 +14810,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_task_planning_fields_round_trip, test_overdue_rules, test_milestone_reward_needs_all_milestones, test_silent_tasks_invisible_without_passcode, test_silent_completion_has_no_celebration_flag, test_migration_defaults_existing_tasks</t>
+          <t>test_task_planning_fields_round_trip, test_overdue_rules, test_due_filters_milestones_and_sort, test_milestone_reward_needs_all_milestones, test_dashboard_overdue_and_milestones, test_migration_defaults_existing_tasks; quiet completion and celebrations verified in the browser; ⏳ test_silent_tasks_invisible_without_passcode comes with the passcode</t>
         </is>
       </c>
     </row>
@@ -17118,7 +17118,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅ (branch; hiding silent tasks from visitors comes with hosting)</t>
         </is>
       </c>
     </row>
@@ -17666,7 +17666,7 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reward ideas and wishlist (HLR-12)
- Ideas: a reward with status "idea" and no rule; quick capture with
  title, for whom, one-tap cover photo, and optional where seen, link,
  note and area. Private (silent) by default
- Turn an idea into a reward (task count or milestone completed),
  keeping its details; close as bought or dropped, and reopen
- For whom on every reward, with suggestions and a filter; ideas in
  search; dashboard counts open ideas per person
- Cover photos stored privately and served by signed links
- Migration 0005_reward_ideas defaults existing rewards to "Me" and
  announced with no data loss
- Separate throwaway test backend and standalone MFE launch configs so
  testing never touches the real app
- Docs and workbook updated; 73 tests pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rewards/Rewards_HLRD_LLRD.xlsx
+++ b/docs/rewards/Rewards_HLRD_LLRD.xlsx
@@ -4467,12 +4467,12 @@
       </c>
       <c r="B181" s="7" t="inlineStr">
         <is>
-          <t>Rewards accept status: "idea" on create (rule, threshold and tile then optional), forWhom, visibility, link, seenAt (where seen) and a cover image; POST /rewards/{id}/activate (rule, threshold, tile, tasks) turns an idea into a locked reward; POST /rewards/{id}/close with outcome (bought | dropped); GET /rewards filters status=idea|closed and forWhom=</t>
+          <t>POST /rewards accepts status: "idea", forWhom, visibility, link and whereSeen; POST /rewards/{id}/activate (ruleType, threshold), /close (outcome: bought | dropped) and /reopen; PUT / DELETE /rewards/{id}/cover (multipart photo; served by a signed link like files); GET /rewards filters status=idea|closed and forWhom=; GET /rewards-people lists everyone for suggestions; ideas can't be linked or claimed (409)</t>
         </is>
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
     <row r="254">
       <c r="A254" s="13" t="inlineStr">
         <is>
-          <t>LLR-12 Reward ideas and wishlist (HLR-12) ⏳ next</t>
+          <t>LLR-12 Reward ideas and wishlist (HLR-12) ✅</t>
         </is>
       </c>
     </row>
@@ -5284,7 +5284,7 @@
     <row r="257">
       <c r="A257" s="13" t="inlineStr">
         <is>
-          <t>LLR-12 Reward ideas and wishlist (HLR-12) ⏳ next</t>
+          <t>LLR-12 Reward ideas and wishlist (HLR-12) ✅</t>
         </is>
       </c>
     </row>
@@ -5313,12 +5313,12 @@
       </c>
       <c r="B259" s="7" t="inlineStr">
         <is>
-          <t>Quick capture: a "+ Idea" button on the Rewards tab and on every tile and area screen opens a short form: title (required, 1–200), then optional for whom, notes (≤ 2000), link (URL), cover photo (camera or gallery, via the file rules of LLR-10.7), where seen (e.g. "City library") and tile/area. Saving needs only the title</t>
+          <t>Quick capture: "💡 + Idea" on the Rewards screen and on every area's Rewards tab opens a short form: title (required), for whom (default Me) and a one-tap cover photo (camera or gallery; JPG, PNG, WebP or HEIC up to 10 MB); *More* adds where seen, link, note and (on the Rewards screen) an optional area. Saving needs only the title</t>
         </is>
       </c>
       <c r="C259" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="C260" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       </c>
       <c r="C261" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5364,12 +5364,12 @@
       </c>
       <c r="B262" s="7" t="inlineStr">
         <is>
-          <t>The Rewards tab has an Ideas filter (and *Closed* for bought or dropped ideas), and can be filtered by for whom, e.g. "Shiragi's ideas and rewards". Tile and area screens list their ideas under "Rewards you can earn here" in a separate *Ideas* group</t>
+          <t>The Rewards screen filters by status (💡 Ideas, Locked, Unlocked, Claimed, Closed) and by for whom (e.g. *Shiragi*), plus search; closed ideas are hidden unless *Closed* is chosen. An area's Rewards tab lists its ideas with its rewards. Ideas are never offered on the Link screen</t>
         </is>
       </c>
       <c r="C262" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5381,12 +5381,12 @@
       </c>
       <c r="B263" s="7" t="inlineStr">
         <is>
-          <t>Turn into a reward: from an idea, add a rule (N completions, streak of N or milestone completed), a threshold, a tile (and optional area) and tasks. It becomes a normal *locked* reward, keeping its title, photo, link, notes and for whom; the unlock check runs straight away (BR-R28)</t>
+          <t>Turn into reward: on an idea, pick how it unlocks (task count with N, or milestone completed). It becomes a normal *locked* reward with the same id, keeping title, photo, link, note, where seen, area and for whom; tasks are then linked on the Link screen (BR-R28)</t>
         </is>
       </c>
       <c r="C263" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="C264" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="C265" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>🟡 private by default with a 🔕 marker; hiding from visitors comes with the owner passcode (hosting)</t>
         </is>
       </c>
     </row>
@@ -5437,7 +5437,7 @@
       </c>
       <c r="C266" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="C267" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="B272" s="7" t="inlineStr">
         <is>
-          <t>Turning an idea into a reward requires a rule, a threshold (except *milestone completed*) and a tile (LLR-4.9); the idea's id is kept, so links and photos stay attached</t>
+          <t>Turning an idea into a reward requires a rule and a threshold (except *milestone completed*); a tile isn't required since rewards stand alone. The idea's id is kept, so links and photos stay attached</t>
         </is>
       </c>
     </row>
@@ -7088,7 +7088,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -11351,12 +11351,12 @@
       </c>
       <c r="D118" s="8" t="inlineStr">
         <is>
-          <t>Rewards accept status: "idea" on create (rule, threshold and tile then optional), forWhom, visibility, link, seenAt (where seen) and a cover image; POST /rewards/{id}/activate (rule, threshold, tile, tasks) turns an idea into a locked reward; POST /rewards/{id}/close with outcome (bought | dropped); GET /rewards filters status=idea|closed and forWhom=</t>
+          <t>POST /rewards accepts status: "idea", forWhom, visibility, link and whereSeen; POST /rewards/{id}/activate (ruleType, threshold), /close (outcome: bought | dropped) and /reopen; PUT / DELETE /rewards/{id}/cover (multipart photo; served by a signed link like files); GET /rewards filters status=idea|closed and forWhom=; GET /rewards-people lists everyone for suggestions; ideas can't be linked or claimed (409)</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F118" s="8" t="inlineStr">
@@ -12495,12 +12495,12 @@
       </c>
       <c r="D144" s="8" t="inlineStr">
         <is>
-          <t>Quick capture: a "+ Idea" button on the Rewards tab and on every tile and area screen opens a short form: title (required, 1–200), then optional for whom, notes (≤ 2000), link (URL), cover photo (camera or gallery, via the file rules of LLR-10.7), where seen (e.g. "City library") and tile/area. Saving needs only the title</t>
+          <t>Quick capture: "💡 + Idea" on the Rewards screen and on every area's Rewards tab opens a short form: title (required), for whom (default Me) and a one-tap cover photo (camera or gallery; JPG, PNG, WebP or HEIC up to 10 MB); *More* adds where seen, link, note and (on the Rewards screen) an optional area. Saving needs only the title</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F144" s="8" t="inlineStr">
@@ -12544,7 +12544,7 @@
       </c>
       <c r="E145" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F145" s="8" t="inlineStr">
@@ -12588,7 +12588,7 @@
       </c>
       <c r="E146" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F146" s="8" t="inlineStr">
@@ -12627,12 +12627,12 @@
       </c>
       <c r="D147" s="8" t="inlineStr">
         <is>
-          <t>The Rewards tab has an Ideas filter (and *Closed* for bought or dropped ideas), and can be filtered by for whom, e.g. "Shiragi's ideas and rewards". Tile and area screens list their ideas under "Rewards you can earn here" in a separate *Ideas* group</t>
+          <t>The Rewards screen filters by status (💡 Ideas, Locked, Unlocked, Claimed, Closed) and by for whom (e.g. *Shiragi*), plus search; closed ideas are hidden unless *Closed* is chosen. An area's Rewards tab lists its ideas with its rewards. Ideas are never offered on the Link screen</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F147" s="8" t="inlineStr">
@@ -12671,12 +12671,12 @@
       </c>
       <c r="D148" s="8" t="inlineStr">
         <is>
-          <t>Turn into a reward: from an idea, add a rule (N completions, streak of N or milestone completed), a threshold, a tile (and optional area) and tasks. It becomes a normal *locked* reward, keeping its title, photo, link, notes and for whom; the unlock check runs straight away (BR-R28)</t>
+          <t>Turn into reward: on an idea, pick how it unlocks (task count with N, or milestone completed). It becomes a normal *locked* reward with the same id, keeping title, photo, link, note, where seen, area and for whom; tasks are then linked on the Link screen (BR-R28)</t>
         </is>
       </c>
       <c r="E148" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F148" s="8" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="E149" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F149" s="8" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="E150" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built (manual test)</t>
         </is>
       </c>
       <c r="F150" s="8" t="inlineStr">
@@ -12808,7 +12808,7 @@
       </c>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F151" s="8" t="inlineStr">
@@ -12852,7 +12852,7 @@
       </c>
       <c r="E152" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F152" s="8" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="E179" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F179" s="8" t="inlineStr">
@@ -14079,12 +14079,12 @@
       </c>
       <c r="D180" s="8" t="inlineStr">
         <is>
-          <t>Turning an idea into a reward requires a rule, a threshold (except *milestone completed*) and a tile (LLR-4.9); the idea's id is kept, so links and photos stay attached</t>
+          <t>Turning an idea into a reward requires a rule and a threshold (except *milestone completed*); a tile isn't required since rewards stand alone. The idea's id is kept, so links and photos stay attached</t>
         </is>
       </c>
       <c r="E180" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F180" s="8" t="inlineStr">
@@ -14128,7 +14128,7 @@
       </c>
       <c r="E181" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F181" s="8" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="E182" s="8" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Built &amp; tested</t>
         </is>
       </c>
       <c r="F182" s="8" t="inlineStr">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>⏳ planned: test_idea_needs_only_title, test_idea_never_unlocks_or_counts, test_activate_idea_keeps_details_and_evaluates, test_close_and_reopen_idea, test_ideas_silent_by_default, test_filter_by_for_whom, test_migration_defaults_existing_rewards</t>
+          <t>test_idea_needs_only_title, test_ideas_silent_by_default, test_idea_never_unlocks_or_counts, test_activate_idea_keeps_details_and_evaluates, test_close_and_reopen_idea, test_filter_by_for_whom, test_cover_photo_signed_link_and_cleanup, test_ideas_in_search, test_migration_defaults_existing_rewards</t>
         </is>
       </c>
     </row>
@@ -17135,7 +17135,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅ (branch; hiding private ideas from visitors comes with hosting)</t>
         </is>
       </c>
     </row>
@@ -17693,7 +17693,7 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>⏳ next</t>
+          <t>✅</t>
         </is>
       </c>
     </row>

</xml_diff>